<commit_message>
Adicionando 3° batch de testes
Rodei as 10 tasks, agora com o Gemini 3.5 flash.
</commit_message>
<xml_diff>
--- a/batch_timed_results.xlsx
+++ b/batch_timed_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,23 +413,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>gemma-4-31b-it</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>gemma-4-26b-a4b-it</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>gemini-3.5-flash-lite</t>
         </is>
       </c>
     </row>
@@ -1069,6 +1062,20 @@
 Tempo: 378.67s</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+0 0 0 0 0 8 8
+8 8 0 0 0 1 8
+8 1 0 0 0 0 0
+0 0 0 8 1 0 0
+0 0 0 8 8 0 0
+1 8 0 0 0 0 0
+8 8 0 0 0 0 0
+&lt;/prediction&gt;
+Tempo: 36.71s</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1510,6 +1517,25 @@
 Tempo: 377.28s</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+0 0 0 0 0 0 0 0 0 0 0 0
+5 5 5 5 5 0 0 5 5 5 5 0
+5 2 2 2 5 0 0 5 5 2 5 0
+5 2 2 2 5 0 0 5 2 2 5 0
+5 2 2 2 5 0 0 5 2 2 5 0
+5 5 5 5 5 0 0 5 5 5 5 0
+0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0
+0 0 5 5 5 5 5 5 0 0 0 0
+0 0 5 2 2 2 2 5 0 0 0 0
+0 0 5 2 2 2 2 5 0 0 0 0
+0 0 5 5 5 5 5 5 0 0 0 0
+&lt;/prediction&gt;
+Tempo: 35.42s</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1622,6 +1648,14 @@
     There are orthogonal connections.
     Output should be 7.
 Tempo: 235.71s</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+1
+&lt;/prediction&gt;
+Tempo: 36.35s</t>
         </is>
       </c>
     </row>
@@ -2132,6 +2166,24 @@
 Tempo: 377.40s</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
+&lt;/prediction&gt;
+Tempo: 35.74s</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2622,6 +2674,18 @@
 Tempo: 376.91s</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+3 0 0 0 0 3 0 0 3 3 3 0 3 0 3 0 3
+0 3 3 0 0 3 0 0 0 3 0 3 3 3 0 0 0
+3 3 3 3 3 0 0 0 3 0 0 0 3 0 0 0 3
+3 0 3 0 3 0 0 0 0 3 3 3 3 3 3 0 3
+0 3 3 0 0 0 0 0 0 0 3 3 3 0 3 3 0
+&lt;/prediction&gt;
+Tempo: 42.96s</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2752,6 +2816,19 @@
 Tempo: 224.67s</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+3 2 3 2 3 2
+7 8 7 8 7 8
+2 3 2 3 2 3
+8 7 8 7 8 7
+3 2 3 2 3 2
+7 8 7 8 7 8
+&lt;/prediction&gt;
+Tempo: 64.38s</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3405,6 +3482,16 @@
     Is it possible the output is:
     3
 Tempo: 396.81s</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+4 7 1
+3 3 7
+6 2 8
+&lt;/prediction&gt;
+Tempo: 39.08s</t>
         </is>
       </c>
     </row>
@@ -3834,6 +3921,28 @@
     Index 8: 0
     Index 9: 0
 Tempo: 377.80s</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+1 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 1 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 1 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 2 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 2 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+&lt;/prediction&gt;
+Tempo: 34.88s</t>
         </is>
       </c>
     </row>
@@ -4448,6 +4557,19 @@
 Tempo: 376.84s</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+0 0 2 2 3 3 
+0 2 0 3 3 0 
+2 0 2 3 0 0 
+0 6 6 0 4 0 
+6 0 6 4 0 4 
+6 6 0 0 4 0 
+&lt;/prediction&gt;
+Tempo: 33.83s</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4662,6 +4784,23 @@
 Tempo: 269.03s</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>&lt;prediction&gt;
+8 9 0 0 0 0 0 0 0 0
+2 4 0 0 0 4 4 0 0 0
+0 0 0 2 2 2 4 0 0 0
+0 0 0 8 2 2 4 0 0 0
+0 0 0 8 9 8 0 0 0 0
+0 0 0 8 8 9 0 0 0 0
+0 0 0 8 9 9 0 0 0 0
+0 0 0 4 9 9 0 0 0 0
+0 0 0 0 0 9 0 0 0 0
+0 0 0 0 0 0 0 0 0 0
+&lt;/prediction&gt;
+Tempo: 37.06s</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4679,6 +4818,11 @@
           <t>3392.92s</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>396.93s</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Corrigindo o 3° batch de testes, já que faltou o Reasoning
</commit_message>
<xml_diff>
--- a/batch_timed_results.xlsx
+++ b/batch_timed_results.xlsx
@@ -1,452 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Desktop\Escola_Trabalho\Faculdade\UFRGS\5°_semestre\PCI\Projeto 1\PCI-GrupoA\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27634165-089C-432E-8984-215144F28B67}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>gemma-4-31b-it</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>gemma-4-26b-a4b-it</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>gemini-3.5-flash-lite</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>3aa6fb7a.json</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>gemma-4-31b-it</t>
+  </si>
+  <si>
+    <t>gemma-4-26b-a4b-it</t>
+  </si>
+  <si>
+    <t>3aa6fb7a.json</t>
+  </si>
+  <si>
+    <t>The user wants me to extract the final predicted grid from the provided reasoning text.
     *   The reasoning text analyzes two examples and a test input.
     *   The rule identified is: find connected groups of three 8s forming an L-shape in a 2x2 block and fill the missing fourth cell with 1.
     *   The test input is:
@@ -521,11 +109,9 @@
     Group 4: (5,1), (6,0), (6,1) -&gt; Missing (5,0)
     Everything seems correct.
 Tempo: 244.16s</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>*   Input: 7x7 grid with 0s and 8s.
+  </si>
+  <si>
+    <t>*   Input: 7x7 grid with 0s and 8s.
     *   Rule: Identify connected components of 8s that form 3/4 of a 2x2 square and fill the 4th cell with a 1.
     *   Input Grid:
         ```
@@ -1060,11 +646,9 @@
         Row 1: 8 8 0 0 0 0 8
         Col
 Tempo: 378.67s</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
 0 0 0 0 0 8 8
 8 8 0 0 0 1 8
 8 1 0 0 0 0 0
@@ -1073,19 +657,14 @@
 1 8 0 0 0 0 0
 8 8 0 0 0 0 0
 &lt;/prediction&gt;
-Tempo: 36.71s</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>44d8ac46.json</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>The user wants me to extract the final predicted grid from the reasoning text.
+Reasoning Summary: The task is to identify L-shapes formed by three `8`s in any $2 \times 2$ subgrid and place a `1` in the remaining empty `0` cell of that $2 \times 2$ block.
+Tempo: 35.70s</t>
+  </si>
+  <si>
+    <t>44d8ac46.json</t>
+  </si>
+  <si>
+    <t>The user wants me to extract the final predicted grid from the reasoning text.
     *   Input grid size: 12x12.
     *   Shape 1: (1,0) to (5,4) - 5x5 rectangle. Hole: (2,1) to (4,3) - 3x3 square.
     *   Shape 2: (1,7) to (5,10) - 5x4 rectangle. Hole: (2,9), (3,8), (3,9), (4,8), (4,9) - irregular.
@@ -1149,11 +728,9 @@
     This is a 2x4 rectangle. Not a square.
     So only Shape 1's hole (3x3) is filled.
 Tempo: 315.47s</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>*   Input: A grid of 0s and 5s.
+  </si>
+  <si>
+    <t>*   Input: A grid of 0s and 5s.
     *   Rule: Identify connected components of 0s that are completely enclosed by 5s. If a component is a solid square (k x k), change its 0s to 2s.
     *   Input Grid:
         ```
@@ -1515,11 +1092,9 @@
         Row 1: 5 5 5 5 (cols 7,8,9,10)
         Row 2: 5 5 0 
 Tempo: 377.28s</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
 0 0 0 0 0 0 0 0 0 0 0 0
 5 5 5 5 5 0 0 5 5 5 5 0
 5 2 2 2 5 0 0 5 5 2 5 0
@@ -1533,19 +1108,15 @@
 0 0 5 2 2 2 2 5 0 0 0 0
 0 0 5 5 5 5 5 5 0 0 0 0
 &lt;/prediction&gt;
-Tempo: 35.42s</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>44f52bb0.json</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>The user wants me to extract the final predicted value from the provided reasoning text.
+Reasoning Summary:
+The task is to identify closed gray rectangular shapes (color 5) and fill their completely enclosed interior regions (which are originally black/0) with red (color 2). Applying this rule to the test input fills the hollow centers of the top-left, top-right, and bottom-left shapes with red pixels.
+Tempo: 35.18s</t>
+  </si>
+  <si>
+    <t>44f52bb0.json</t>
+  </si>
+  <si>
+    <t>The user wants me to extract the final predicted value from the provided reasoning text.
 The reasoning text analyzes several examples of 3x3 grids containing 0s and 2s and their corresponding outputs (1 or 7).
 The reasoning concludes that the rule is based on vertical symmetry (Column 1 = Column 3).
 The test input is:
@@ -1555,11 +1126,9 @@
 Column 1 is [2, 2, 2] and Column 3 is [2, 2, 2].
 Since they are identical, the predicted output is 1.
 Tempo: 186.48s</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>*   Example 1: 5 cells, 0 ortho connections, 1 diag component (all connected) -&gt; Output 1
+  </si>
+  <si>
+    <t>*   Example 1: 5 cells, 0 ortho connections, 1 diag component (all connected) -&gt; Output 1
     *   Example 2: 3 cells, 1 ortho connection, 1 diag component (all connected) -&gt; Output 7
     *   Example 3: 6 cells, 4 ortho connections, 2 diag components (not all connected) -&gt; Output 1
     *   Example 4: 2 cells, 0 ortho connections, 2 diag components (not all connected) -&gt; Output 1
@@ -1648,26 +1217,20 @@
     There are orthogonal connections.
     Output should be 7.
 Tempo: 235.71s</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
-1
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
+7
 &lt;/prediction&gt;
-Tempo: 36.35s</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>0a938d79.json</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>*   Input grid: 11 rows, 27 columns.
+**Reasoning Summary:** 
+By analyzing the examples and counting the number of red pixels (`2`) in the input grids, we observe that the output scalar corresponds to specific properties of the red pixel count or layout. Specifically, the test input contains 7 red pixels arranged in a symmetrical H-like pattern, and matching the logic from the examples (such as Example 2 where a count of 3 yields output `7`), the final predicted scalar value is `7`.
+Tempo: 36.14s</t>
+  </si>
+  <si>
+    <t>0a938d79.json</t>
+  </si>
+  <si>
+    <t>*   Input grid: 11 rows, 27 columns.
     *   P1 = (0, 5), v1 = 3.
     *   P2 = (10, 10), v2 = 4.
     *   P1 is on the top edge (r=0), so the stripes are vertical.
@@ -1699,11 +1262,9 @@
         Col 26: 0 (1 zero)
         Total columns: 5 (0-4) + 1 (5) + 4 (6-9) + 1 (10) + 4 (11-14) + 1 (15) + 4 (16-19) + 1 (20) + 4 (21-24) + 1 (25) + 1 (26) = 27. Correct.
 Tempo: 380.39s</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>*   Input: 11x27 grid.
+  </si>
+  <si>
+    <t>*   Input: 11x27 grid.
     *   Non-zero elements:
         *   Color 1: 5 at (0, 1)
         *   Color 2: 2 at (10, 11)
@@ -2164,11 +1725,9 @@
         Yes.
         Wait, let me re-check the row content
 Tempo: 377.40s</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
 0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
 0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
 0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
@@ -2181,19 +1740,14 @@
 0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
 0 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0 0 0 0 4 0 0 0 0 3 0
 &lt;/prediction&gt;
-Tempo: 35.74s</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>0b148d64.json</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+Reasoning Summary: The input contains colored pixels at `(0, 5) = 3` and `(10, 10) = 4`. Following a column-based periodic propagation with a spacing of 5 columns (the difference between 10 and 5), the colors 3 and 4 extend vertically down all rows and repeat horizontally every 5 columns across the grid width.
+Tempo: 37.53s</t>
+  </si>
+  <si>
+    <t>0b148d64.json</t>
+  </si>
+  <si>
+    <t>The user wants me to extract the final predicted grid from the provided reasoning text.
     *   The reasoning text identifies the pattern: the input grid is divided into four sections. Three sections have the same color, and one has a unique color. The output is the section with the unique color.
     *   For the test input:
         *   Top-left: Color 1 (blue)
@@ -2217,11 +1771,9 @@
     *   The output should be only the &lt;prediction&gt; tags containing the numbers.
     *   No explanations or conversational text.
 Tempo: 232.58s</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>*   Input: 15x17 grid.
+  </si>
+  <si>
+    <t>*   Input: 15x17 grid.
     *   Rows 0-5: Contains colors 1 and 3.
     *   Rows 6-9: All 0s.
     *   Rows 10-14: Contains only color 3.
@@ -2672,30 +2224,29 @@
         3 (col 0)
         0 (col 
 Tempo: 376.91s</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
-3 0 0 0 0 3 0 0 3 3 3 0 3 0 3 0 3
-0 3 3 0 0 3 0 0 0 3 0 3 3 3 0 0 0
-3 3 3 3 3 0 0 0 3 0 0 0 3 0 0 0 3
-3 0 3 0 3 0 0 0 0 3 3 3 3 3 3 0 3
-0 3 3 0 0 0 0 0 0 0 3 3 3 0 3 3 0
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
+3 3 3 0 3 0 3 0 3
+0 3 0 3 3 3 0 0 0
+0 0 0 3 3 3 3 0 0
+3 3 0 3 3 0 3 0 0
+0 3 0 3 3 3 0 3 3
+3 3 0 0 0 3 0 0 3
+3 3 3 0 3 0 3 0 3
+0 3 0 3 3 3 0 0 0
+3 0 0 0 3 0 0 0 3
+0 3 3 3 3 3 3 0 3
+0 0 3 3 3 0 3 3 0
 &lt;/prediction&gt;
-Tempo: 42.96s</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>00576224.json</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>*   Input: 2x2 grid `[[3, 2], [7, 8]]`
+Reasoning Summary: The task requires extracting the second non-zero sub-grid (the right-hand side pattern) from the input, which is composed of color 3, and outputting its exact shape and values.
+Tempo: 35.30s</t>
+  </si>
+  <si>
+    <t>00576224.json</t>
+  </si>
+  <si>
+    <t>*   Input: 2x2 grid `[[3, 2], [7, 8]]`
     *   Rule:
         *   Row 1: Input Row 1 repeated 3 times (`3 2 3 2 3 2`)
         *   Row 2: Input Row 2 repeated 3 times (`7 8 7 8 7 8`)
@@ -2711,11 +2262,9 @@
         3 2 3 2 3 2
         7 8 7 8 7 8
 Tempo: 194.39s</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>*   Input:
+  </si>
+  <si>
+    <t>*   Input:
         ```
         3 2
         7 8
@@ -2814,11 +2363,9 @@
     Row 5: 7 8 7 8 7 8
     Looks solid.
 Tempo: 224.67s</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
 3 2 3 2 3 2
 7 8 7 8 7 8
 2 3 2 3 2 3
@@ -2826,19 +2373,14 @@
 3 2 3 2 3 2
 7 8 7 8 7 8
 &lt;/prediction&gt;
-Tempo: 64.38s</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>0a1d4ef5.json</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>The user wants me to extract the final predicted grid or scalar value from the provided reasoning text.
+Reasoning Summary: The 2x2 input is expanded into a 6x6 grid by tiling it in a 3x3 macro-grid where the blocks alternate between the normal input and its horizontally flipped version in the row pattern: Normal, Normal, Normal / Flipped, Flipped, Flipped / Normal, Normal, Normal.
+Tempo: 34.83s</t>
+  </si>
+  <si>
+    <t>0a1d4ef5.json</t>
+  </si>
+  <si>
+    <t>The user wants me to extract the final predicted grid or scalar value from the provided reasoning text.
     *   The reasoning text identifies blocks of colors in a 30x30 grid.
     *   It finds 4 rows of 3 blocks each.
     *   Row 1: 2, 3, 3
@@ -2853,11 +2395,9 @@
     *   The output must be only the &lt;prediction&gt; tags containing the numbers.
     *   No explanations or conversational text.
 Tempo: 266.02s</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>*   The goal is to extract the final predicted grid or scalar value from the reasoning text.
+  </si>
+  <si>
+    <t>*   The goal is to extract the final predicted grid or scalar value from the reasoning text.
     *   The reasoning text is incomplete (it ends abruptly).
     *   Wait, the reasoning text *ends* with "3:". It doesn't provide the final answer for Example 3.
     *   Let me re-read the reasoning text.
@@ -3482,28 +3022,21 @@
     Is it possible the output is:
     3
 Tempo: 396.81s</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
+5 3 8
 4 7 1
-3 3 7
-6 2 8
+4 6 2
 &lt;/prediction&gt;
-Tempo: 39.08s</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>0b17323b.json</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>*   Input: 15x15 grid.
+Reasoning Summary: The output is a $3 \times 3$ grid representing the spatial arrangement (Top-Left, Top-Center, Top-Right, Middle-Left, Center, Middle-Right, Bottom-Left, Bottom-Center, Bottom-Right) of the distinct colored blocks found within the input grid.
+Tempo: 36.28s</t>
+  </si>
+  <si>
+    <t>0b17323b.json</t>
+  </si>
+  <si>
+    <t>*   Input: 15x15 grid.
     *   '1' positions: (0, 0), (3, 3), (6, 6).
     *   Pattern: Constant difference (delta_row, delta_col) = (3, 3).
     *   Sequence: (0, 0), (3, 3), (6, 6), (9, 9), (12, 12).
@@ -3546,11 +3079,9 @@
     *   '2's at (9,9), (12,12)? Yes.
     *   All others 0? Yes.
 Tempo: 170.22s</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>*   Input: 15x15 grid with blue (1) pixels at (0,0), (3,3), (6,6).
+  </si>
+  <si>
+    <t>*   Input: 15x15 grid with blue (1) pixels at (0,0), (3,3), (6,6).
     *   Pattern: The blue pixels follow a step of (3,3).
     *   Rule: Continue the pattern with red (2) pixels.
     *   Next pixels in pattern:
@@ -3921,11 +3452,9 @@
     Index 8: 0
     Index 9: 0
 Tempo: 377.80s</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
 1 0 0 0 0 0 0 0 0 0 0 0 0 0 0
 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
@@ -3942,19 +3471,14 @@
 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
 &lt;/prediction&gt;
-Tempo: 34.88s</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>0bb8deee.json</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+Reasoning Summary: The task requires continuing a diagonal sequence of blue pixels (`1`) which are spaced by a step of $(+3, +3)$ starting from $(0, 0)$, $(3, 3)$, and $(6, 6)$. Red pixels (`2`) are then placed following the exact same step pattern at $(9, 9)$ and $(12, 12)$ until reaching the grid boundaries.
+Tempo: 49.83s</t>
+  </si>
+  <si>
+    <t>0bb8deee.json</t>
+  </si>
+  <si>
+    <t>The user wants me to extract the final predicted grid from the provided reasoning text.
 Looking at the reasoning text:
 - The final combined 6x6 grid is:
   0 2 2 3 3 3
@@ -3965,11 +3489,9 @@
   6 6 0 0 4 0
 I need to output this grid inside `&lt;prediction&gt;` tags.
 Tempo: 249.02s</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>*   The task is to extract the final predicted grid or scalar value from the reasoning text.
+  </si>
+  <si>
+    <t>*   The task is to extract the final predicted grid or scalar value from the reasoning text.
     *   The reasoning text describes a pattern where a grid is divided by a divider (a row and a column of the same color).
     *   The four quadrants each contain a shape.
     *   The output is a 6x6 grid formed by placing the 3x3 bounding boxes of these four shapes into a 2x2 arrangement.
@@ -4555,31 +4077,25 @@
     *   (Analysis of Example 3)
     *   Wait, I'm
 Tempo: 376.84s</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
-0 0 2 2 3 3 
-0 2 0 3 3 0 
-2 0 2 3 0 0 
-0 6 6 0 4 0 
-6 0 6 4 0 4 
-6 6 0 0 4 0 
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
+0 0 0 0 0 0 0 0 3 3 3 0
+0 0 2 2 0 0 0 0 0 3 3 0
+0 0 2 0 0 0 0 0 3 0 0 0
+0 2 0 2 0 0 0 0 0 0 0 0
+0 0 6 6 0 0 0 0 0 4 0 0
+0 6 0 6 0 0 0 0 4 0 4 0
+0 6 6 0 0 0 0 0 0 4 0 0
 &lt;/prediction&gt;
-Tempo: 33.83s</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>0becf7df.json</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+Reasoning Summary: The input grid is partitioned into four quadrants by intersecting horizontal and vertical lines. The output is formed by removing the dividing lines and combining the four quadrant shapes adjacently into a single compact grid (top-left paired with top-right, and bottom-left paired with bottom-right).
+Tempo: 35.25s</t>
+  </si>
+  <si>
+    <t>0becf7df.json</t>
+  </si>
+  <si>
+    <t>The user wants me to extract the final predicted grid from the provided reasoning text.
     *   The reasoning text describes a pattern based on three examples.
     *   The pattern involves a 2x2 block at the top-left corner.
     *   The colors in the first row (C1, C2) and second row (C3, C4) of this 2x2 block are swapped (C1 &lt;-&gt; C2 and C3 &lt;-&gt; C4) for all other cells in the grid.
@@ -4678,11 +4194,9 @@
     0 0 0 0 0 2 0 0 0 0
     0 0 0 0 0 0 0 0 0 0
 Tempo: 327.94s</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>*   Input: A 10x10 grid with non-zero values.
+  </si>
+  <si>
+    <t>*   Input: A 10x10 grid with non-zero values.
     *   Task: Identify the pattern and predict the output grid.
     *   Pattern identified:
         1.  The top-left 2x2 block defines two color pairs: `(color at (0,0), color at (0,1))` and `(color at (1,0), color at (1,1))`.
@@ -4782,46 +4296,555 @@
         0 0 0 0 0 0 0 0 0 0
         Looks solid.
 Tempo: 269.03s</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>&lt;prediction&gt;
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
 8 9 0 0 0 0 0 0 0 0
-2 4 0 0 0 4 4 0 0 0
-0 0 0 2 2 2 4 0 0 0
-0 0 0 8 2 2 4 0 0 0
-0 0 0 8 9 8 0 0 0 0
-0 0 0 8 8 9 0 0 0 0
-0 0 0 8 9 9 0 0 0 0
-0 0 0 4 9 9 0 0 0 0
-0 0 0 0 0 9 0 0 0 0
+2 4 0 0 0 8 8 0 0 0
+0 0 0 9 9 9 8 0 0 0
+0 0 0 4 9 9 8 0 0 0
+0 0 0 4 2 4 0 0 0 0
+0 0 0 4 4 2 0 0 0 0
+0 0 0 4 2 2 0 0 0 0
+0 0 0 8 2 2 0 0 0 0
+0 0 0 0 0 2 0 0 0 0
 0 0 0 0 0 0 0 0 0 0
 &lt;/prediction&gt;
-Tempo: 37.06s</t>
-        </is>
+Reasoning Summary:
+The top-left 2x2 subgrid defines pairwise color swaps based on its rows: the two colors in the first row swap with each other, and the two colors in the second row swap with each other. For the test input, the top-left 2x2 is `8 9 / 2 4`, meaning `8` and `9` swap, and `2` and `4` swap throughout the entire grid, while the top-left 2x2 itself remains unchanged.
+Tempo: 37.65s</t>
+  </si>
+  <si>
+    <t>Tempo do Batch</t>
+  </si>
+  <si>
+    <t>2567.28s</t>
+  </si>
+  <si>
+    <t>3392.92s</t>
+  </si>
+  <si>
+    <t>374.31s</t>
+  </si>
+  <si>
+    <t>gemini-3.5-flash-lite (max tokens igual)</t>
+  </si>
+</sst>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Tempo do Batch</t>
-        </is>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2567.28s</t>
-        </is>
+      <c r="B2" t="s">
+        <v>4</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>3392.92s</t>
-        </is>
+      <c r="C2" t="s">
+        <v>5</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>396.93s</t>
-        </is>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicionando 4° batch de testes e análises realizadas sobre os resultados
Também adicionei o gerador de gráficos (específico, por enquanto, pro caso atual - em outro momento peço pro Gemini criar uma forma mais genérica), e, então, adicionei o necessário pra rodar esse código nos requirements.
</commit_message>
<xml_diff>
--- a/batch_timed_results.xlsx
+++ b/batch_timed_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Desktop\Escola_Trabalho\Faculdade\UFRGS\5°_semestre\PCI\Projeto 1\PCI-GrupoA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27634165-089C-432E-8984-215144F28B67}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DCEBE47-49ED-4874-9831-E4B9B36379A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>Task</t>
   </si>
@@ -29,6 +29,9 @@
   </si>
   <si>
     <t>gemma-4-26b-a4b-it</t>
+  </si>
+  <si>
+    <t>gemini-3.5-flash-lite</t>
   </si>
   <si>
     <t>3aa6fb7a.json</t>
@@ -661,6 +664,19 @@
 Tempo: 35.70s</t>
   </si>
   <si>
+    <t>&lt;prediction&gt;
+0 0 0 0 0 8 8
+8 8 0 0 0 1 8
+8 1 0 0 0 0 0
+0 0 0 8 1 0 0
+0 0 0 8 8 0 0
+1 8 0 0 0 0 0
+8 8 0 0 0 0 0
+&lt;/prediction&gt;
+Reasoning Summary: The rule identifies incomplete $2 \times 2$ blocks containing three teal (8) pixels and one empty (0) pixel, then fills the empty cell with a blue (1) pixel to complete the $2 \times 2$ square.
+Tempo: 35.57s</t>
+  </si>
+  <si>
     <t>44d8ac46.json</t>
   </si>
   <si>
@@ -1113,6 +1129,24 @@
 Tempo: 35.18s</t>
   </si>
   <si>
+    <t>Reasoning Summary: The transformation rule is to fill the interior (enclosed zero-valued cells) of closed gray rectangular shapes with red (color 2). Applying this rule to the test input yields the filled shapes.
+&lt;prediction&gt;
+0 0 0 0 0 0 0 0 0 0 0 0
+5 5 5 5 5 0 0 5 5 5 5 0
+5 2 2 2 5 0 0 5 2 2 5 0
+5 2 2 2 5 0 0 5 2 2 5 0
+5 2 2 2 5 0 0 5 2 2 5 0
+5 5 5 5 5 0 0 5 5 5 5 0
+0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0
+0 0 5 5 5 5 5 5 0 0 0 0
+0 0 5 2 2 2 2 5 0 0 0 0
+0 0 5 2 2 2 2 5 0 0 0 0
+0 0 5 5 5 5 5 5 0 0 0 0
+&lt;/prediction&gt;
+Tempo: 34.31s</t>
+  </si>
+  <si>
     <t>44f52bb0.json</t>
   </si>
   <si>
@@ -1225,6 +1259,13 @@
 **Reasoning Summary:** 
 By analyzing the examples and counting the number of red pixels (`2`) in the input grids, we observe that the output scalar corresponds to specific properties of the red pixel count or layout. Specifically, the test input contains 7 red pixels arranged in a symmetrical H-like pattern, and matching the logic from the examples (such as Example 2 where a count of 3 yields output `7`), the final predicted scalar value is `7`.
 Tempo: 36.14s</t>
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
+7
+&lt;/prediction&gt;
+Reasoning Summary: The rule is to count the total number of red pixels (`2`) in the input grid. If the count is even, the output is `1`. If the count is odd, the output is `7`. Since the test input contains 7 red pixels (an odd number), the output is `7`.
+Tempo: 56.07s</t>
   </si>
   <si>
     <t>0a938d79.json</t>
@@ -1744,6 +1785,23 @@
 Tempo: 37.53s</t>
   </si>
   <si>
+    <t>&lt;prediction&gt;
+3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3 3
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4 4
+&lt;/prediction&gt;
+Reasoning Summary: The transformation identifies seed pixels at specific rows and fills their respective rows entirely across the grid width based on the vertical positions of the seeds.
+Tempo: 36.08s</t>
+  </si>
+  <si>
     <t>0b148d64.json</t>
   </si>
   <si>
@@ -2243,6 +2301,17 @@
 Tempo: 35.30s</t>
   </si>
   <si>
+    <t>&lt;prediction&gt;
+3 0 0 0 0 3 0 0 3 3 3 0 3 0 3 0 3
+0 3 3 0 0 3 0 0 0 3 0 3 3 3 0 0 0
+3 3 3 3 3 0 0 0 3 0 0 0 3 0 0 0 3
+3 0 3 0 3 0 0 0 0 3 3 3 3 3 3 0 3
+0 3 3 0 0 0 0 0 0 0 3 3 3 0 3 3 0
+&lt;/prediction&gt;
+Reasoning Summary: The task requires isolating and extracting a specific target sub-grid of a secondary color (`3`) from the test input grid, based on patterns established in the training examples.
+Tempo: 35.98s</t>
+  </si>
+  <si>
     <t>00576224.json</t>
   </si>
   <si>
@@ -2377,6 +2446,19 @@
 Tempo: 34.83s</t>
   </si>
   <si>
+    <t>&lt;prediction&gt;
+3 2 3 2 3 2
+7 8 7 8 7 8
+2 3 2 3 2 3
+8 7 8 7 8 7
+3 2 3 2 3 2
+7 8 7 8 7 8
+&lt;/prediction&gt;
+Reasoning Summary:
+The input $2 \times 2$ grid is tiled into a $3 \times 3$ macro-grid to form a $6 \times 6$ output grid. The original block is repeated normally in the 1st and 3rd macro-rows, while the middle (2nd) macro-row consists of the $2 \times 2$ block with its columns horizontally swapped.
+Tempo: 51.77s</t>
+  </si>
+  <si>
     <t>0a1d4ef5.json</t>
   </si>
   <si>
@@ -3031,6 +3113,16 @@
 &lt;/prediction&gt;
 Reasoning Summary: The output is a $3 \times 3$ grid representing the spatial arrangement (Top-Left, Top-Center, Top-Right, Middle-Left, Center, Middle-Right, Bottom-Left, Bottom-Center, Bottom-Right) of the distinct colored blocks found within the input grid.
 Tempo: 36.28s</t>
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
+8 5 8
+4 7 1
+3 6 2
+&lt;/prediction&gt;
+**Reasoning Summary:** 
+The task requires mapping the spatial arrangement of the 9 distinct large rectangular colored blocks in the input grid into a compressed $3 \times 3$ output grid. By scanning the test input's 2D regions (top-left to bottom-right), we extract the representative color of each major block: top-left is 8, top-middle is 5, top-right is 8, middle-left is 4, center is 7, middle-right is 1, bottom-left is 3, bottom-middle is 6, and bottom-right is 2. This forms the resulting $3 \times 3$ grid.
+Tempo: 35.36s</t>
   </si>
   <si>
     <t>0b17323b.json</t>
@@ -3473,6 +3565,27 @@
 &lt;/prediction&gt;
 Reasoning Summary: The task requires continuing a diagonal sequence of blue pixels (`1`) which are spaced by a step of $(+3, +3)$ starting from $(0, 0)$, $(3, 3)$, and $(6, 6)$. Red pixels (`2`) are then placed following the exact same step pattern at $(9, 9)$ and $(12, 12)$ until reaching the grid boundaries.
 Tempo: 49.83s</t>
+  </si>
+  <si>
+    <t>&lt;prediction&gt;
+1 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 1 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 1 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 2 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 2 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+0 0 0 0 0 0 0 0 0 0 0 0 0 0 0
+&lt;/prediction&gt;
+Reasoning Summary: The task requires identifying the diagonal step formed by the input blue pixels (1) and continuing this diagonal line using red pixels (2) starting from the last blue pixel until the edge of the 15x15 grid is reached. For the test input, the blue pixels are at `(0,0)`, `(3,3)`, and `(6,6)`, which follows a step of `(+3, +3)`. Continuing this step yields red pixels at `(9, 9)` and `(12, 12)`.
+Tempo: 58.95s</t>
   </si>
   <si>
     <t>0bb8deee.json</t>
@@ -4092,6 +4205,18 @@
 Tempo: 35.25s</t>
   </si>
   <si>
+    <t>&lt;prediction&gt;
+0 2 2 3 3 3
+2 0 2 0 3 3
+0 2 0 3 0 0
+6 6 0 0 4 0
+6 0 6 4 0 4
+6 6 0 0 4 0
+&lt;/prediction&gt;
+Reasoning Summary: The input grid is divided into four quadrants by a cross-shaped dividing line. The non-zero shapes from each of the four quadrants are extracted and combined side-by-side into a compact 6x6 output grid (top-left and top-right in the upper rows, bottom-left and bottom-right in the lower rows).
+Tempo: 34.19s</t>
+  </si>
+  <si>
     <t>0becf7df.json</t>
   </si>
   <si>
@@ -4315,6 +4440,22 @@
 Tempo: 37.65s</t>
   </si>
   <si>
+    <t>&lt;prediction&gt;
+8 9 0 0 0 0 0 0 0 0
+2 4 0 0 0 4 4 0 0 0
+0 0 0 2 2 2 4 0 0 0
+0 0 0 8 2 2 4 0 0 0
+0 0 0 8 9 8 0 0 0 0
+0 0 0 8 8 9 0 0 0 0
+0 0 0 8 9 9 0 0 0 0
+0 0 0 4 9 9 0 0 0 0
+0 0 0 0 0 9 0 0 0 0
+0 0 0 0 0 0 0 0 0 0
+&lt;/prediction&gt;
+Reasoning Summary: The transformation rule is to use the $2 \times 2$ color-mapping key in the top-left corner of the grid to swap specific pairs of colors within the shape on the right. For the test input, the key specifies the swaps $8 \leftrightarrow 2$ and $9 \leftrightarrow 4$. Applying these color replacements to the right-hand shape yields the final predicted grid.
+Tempo: 36.97s</t>
+  </si>
+  <si>
     <t>Tempo do Batch</t>
   </si>
   <si>
@@ -4327,23 +4468,18 @@
     <t>374.31s</t>
   </si>
   <si>
-    <t>gemini-3.5-flash-lite (max tokens igual)</t>
+    <t>415.76s</t>
+  </si>
+  <si>
+    <t>gemini-3.5-flash-lite  (metade max tokens)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -4371,9 +4507,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4676,10 +4811,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4690,161 +4825,197 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
         <v>47</v>
       </c>
+      <c r="E10" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>57</v>
+      </c>
+      <c r="E12" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>